<commit_message>
Re-export Kahoot set: 15 picked questions, bank-driven generator
build.py now holds the full 22-question bank keyed by bank number, with a
PICKED list selecting what exports, so a different selection is a one-line
change. Time limits come from difficulty and the character-limit check now
fails the build instead of only reporting.

Exported selection: 1, 3, 4, 5, 6, 8, 10, 11, 12, 13, 14, 15, 16, 20, 21.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2zDpHEjjhiN7Qvobfiizh
</commit_message>
<xml_diff>
--- a/kahoot-export/load-balancing-kahoot-15.xlsx
+++ b/kahoot-export/load-balancing-kahoot-15.xlsx
@@ -518,60 +518,60 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Which is NOT one of the three ways one server fails you?</t>
+          <t>“Scale up” (vertical) means...</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Capacity</t>
+          <t>Move from 4 vCPU to 64 vCPU</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Availability</t>
+          <t>Run 16 pods of 4 vCPU each</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Operability</t>
+          <t>Add a second region</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Compatibility</t>
+          <t>Put a CDN in front</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
         <v>20</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>“Scale up” (vertical) means...</t>
+          <t>Health checks decide who is allowed. What does the algorithm decide?</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Move from 4 vCPU to 64 vCPU</t>
+          <t>Which of the allowed backends gets this request</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Run 16 pods of 4 vCPU each</t>
+          <t>Whether the pod is alive</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Add a second region</t>
+          <t>How long the DNS TTL is</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Put a CDN in front</t>
+          <t>Which region the user hits</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -617,27 +617,27 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Which algorithm gives you session affinity?</t>
+          <t>Round robin picks a backend by...</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>IP hash</t>
+          <t>The order requests arrive - whose turn is it</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Round robin</t>
+          <t>Live CPU usage</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Least connections</t>
+          <t>The client's IP</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Weighted round robin</t>
+          <t>Response size</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -650,31 +650,31 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Which header carries the real client IP through an L7 balancer?</t>
+          <t>To the backend, a load balancer looks like...</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>X-Forwarded-For</t>
+          <t>The client</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Host</t>
+          <t>The server</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>User-Agent</t>
+          <t>A DNS resolver</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>X-Request-ID</t>
+          <t>A router</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>1</v>
@@ -815,27 +815,27 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Which can an L7 balancer do that an L4 balancer cannot?</t>
+          <t>What does a DNS-based GSLB never see?</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Re-send a failed request to another pod</t>
+          <t>How loaded a region is</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Preserve the client IP</t>
+          <t>Whether a region is up</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Terminate TLS</t>
+          <t>Roughly where the resolver is</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Hold a static IP</t>
+          <t>Your routing policy</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
@@ -848,27 +848,27 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Why does a CDN help an API even at a 0% cache hit rate?</t>
+          <t>Which can an L7 balancer do that an L4 balancer cannot?</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>TCP and TLS handshakes finish ~30 ms away, not ~230 ms</t>
+          <t>Re-send a failed request to another pod</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>It compresses the JSON</t>
+          <t>Preserve the client IP</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>It caches the errors</t>
+          <t>Terminate TLS</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>It lowers origin CPU</t>
+          <t>Hold a static IP</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -881,31 +881,31 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Which clear-text signal lets an L4 balancer route per domain while holding no TLS keys?</t>
+          <t>Why does a CDN help an API even at a 0% cache hit rate?</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SNI in the TLS handshake</t>
+          <t>TCP and TLS handshakes finish ~30 ms away, not ~230 ms</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>The Host header</t>
+          <t>It compresses the JSON</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>X-Forwarded-For</t>
+          <t>It caches the errors</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>The ALPN response</t>
+          <t>It lowers origin CPU</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>1</v>
@@ -988,44 +988,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="96" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="92" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Play order</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
+          <t>Bank #</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
           <t>Difficulty</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Slide</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Correct answer</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
@@ -1035,27 +1041,30 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>slide 6</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Pick one healthy backend from a pool</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Health checks decide who is allowed; the algorithm picks which one. TLS, compression and WAF are features of the box, not of load balancing.</t>
         </is>
@@ -1065,29 +1074,32 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>slide 4</t>
-        </is>
-      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Compatibility</t>
+          <t>slide 10</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Capacity is how much you can serve. Availability is surviving change you did not ask for. Operability is making change you did ask for, safely.</t>
+          <t>Move from 4 vCPU to 64 vCPU</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Scaling up needs no code change but has a ceiling and one power cord. Scaling out survives a dead pod, but needs a balancer in front and an app that keeps no state in memory.</t>
         </is>
       </c>
     </row>
@@ -1095,57 +1107,63 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>slide 10</t>
-        </is>
-      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Move from 4 vCPU to 64 vCPU</t>
+          <t>slide 6</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Scaling up needs no code change but has a ceiling and one power cord. Scaling out survives a dead pod, but needs a balancer in front and an app that keeps no state in memory.</t>
+          <t>Which of the allowed backends gets this request</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Two separate mechanisms. A pod failing its health check is out of the pool entirely, so the algorithm only ever chooses among the survivors.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>slides 13-14</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>IP address and TCP/UDP port</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>It chooses once, at the SYN, and writes (src ip, src port, dst ip, dst port) -&gt; pod into a flow table. Packets 2..N carry no routing hint, so that table is the only memory of the choice.</t>
         </is>
@@ -1153,89 +1171,98 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>slides 38, 41</t>
-        </is>
-      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>IP hash</t>
+          <t>slide 35</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>hash(ip) % N sends the same client to the same server every time, with no table to store. It is the only one of the four that gives affinity, and the only one that ignores load entirely.</t>
+          <t>The order requests arrive - whose turn is it</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>One counter: servers[i++ % N]. It ignores how long each request takes - a 3 s export and a 5 ms health check are both “one turn”.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>slide 7</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>X-Forwarded-For</t>
-        </is>
-      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>The balancer terminates the client connection, so the backend's socket only ever shows the balancer's IP. X-Forwarded-For is the L7 convention for carrying the original.</t>
+          <t>The client</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>To the client the balancer is the server; to the backend it is the client. The backend sees the balancer's IP, so the real one has to be passed in X-Forwarded-For (L7) or PROXY protocol (L4).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>slide 17</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>One 2 s DB blip fails every pod at once</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>A shared dependency inside the check turns “degraded” into “100% down”: every pod fails at the same moment and the pool empties. Keep the check shallow.</t>
         </is>
@@ -1243,29 +1270,32 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>slide 37</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>It has 0 connections and gets flooded</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Zero active connections looks like “completely idle”, so it wins every comparison until it catches up. The fix is slow start: ramp it in instead.</t>
         </is>
@@ -1273,29 +1303,32 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>slides 39-40</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Move sessions to Redis so any pod can serve any user</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Affinity only hides the problem: the pod still holds the cart, so replacing it during a deploy still loses it. IP hash also re-maps ~75% of users when the pod count changes (the rehashing problem, ch. 5). Alex Xu's fix in ch. 1 is shared session storage and a stateless web tier. Keep affinity afterwards only as a cache hint: losing it should cost a cache miss, not a logout.</t>
         </is>
@@ -1303,29 +1336,32 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>slide 27</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Withdrawing the BGP announcement</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Many sites announce the same prefix. Withdraw one and the internet re-learns the next-best path in seconds. No client needs a new answer, because the address never changed.</t>
         </is>
@@ -1333,119 +1369,131 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>slides 14-16</t>
-        </is>
-      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Re-send a failed request to another pod</t>
+          <t>slide 25</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>The L7 proxy still holds the request bytes in memory, so it can write them to a second pod. L4 forwards each packet and forgets it, so there is nothing to replay. An NLB with a TLS listener does terminate TLS, which is what makes that option tempting.</t>
+          <t>How loaded a region is</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Its only inputs are the resolver IP and EDNS Client Subnet, its own health probes, a precomputed latency table, and your policy. A health check answers “is it up”, not “can it take more”, so a saturated healthy region keeps its full share.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>standard</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>slide 28</t>
-        </is>
-      </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>TCP and TLS handshakes finish ~30 ms away, not ~230 ms</t>
+          <t>slides 14-16</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>The edge PoP completes the connection itself, then forwards over a warm pooled connection on a private backbone. That handshake win lands even on requests that can never be cached.</t>
+          <t>Re-send a failed request to another pod</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>The L7 proxy still holds the request bytes in memory, so it can write them to a second pod. L4 forwards each packet and forgets it, so there is nothing to replay. An NLB with a TLS listener does terminate TLS, which is what makes that option tempting.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>hard</t>
-        </is>
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>16</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>slide 14</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>SNI in the TLS handshake</t>
+          <t>slide 28</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>SNI travels in the clear during the handshake, so an L4 balancer can read the hostname without decrypting anything. The Host header sits inside the encrypted stream, and reading that means terminating TLS, which makes you an L7 balancer.</t>
+          <t>TCP and TLS handshakes finish ~30 ms away, not ~230 ms</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>The edge PoP completes the connection itself, then forwards over a warm pooled connection on a private backbone. That handshake win lands even on requests that can never be cached.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>hard</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>double</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>slide 16</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Past the cap it keeps no copy, so there is nothing to re-send</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Retries exist only because the request sits in the proxy's memory. 10,000 concurrent requests x 64 KB is already 640 MB, so every balancer caps what it will buffer. Over the cap it streams the bytes straight through and retries quietly stop working.</t>
         </is>
@@ -1453,29 +1501,32 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>hard</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>double</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>slide 32</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Failover moves traffic, not capacity, so size each region for the whole world: 200,000 / 25,000 = 8. Then lose 1 AZ of 3, x 1.5 = 12. They normally sit at ~33% of rated load, and that idle headroom is what makes failover a non-event.</t>
         </is>

</xml_diff>

<commit_message>
Make Q6 distractors the other three algorithms' criteria
Round robin's options were "live CPU / client IP / response size", two of
which no balancer offers. All four now name a real criterion - least
connections, weighted round robin, IP hash - so the question tests which one
round robin actually uses.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2zDpHEjjhiN7Qvobfiizh
</commit_message>
<xml_diff>
--- a/kahoot-export/load-balancing-kahoot-15.xlsx
+++ b/kahoot-export/load-balancing-kahoot-15.xlsx
@@ -622,22 +622,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The order requests arrive - whose turn is it</t>
+          <t>Whose turn it is in a fixed rotation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Live CPU usage</t>
+          <t>Which server has the fewest active connections</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>The client's IP</t>
+          <t>A weight you set per server</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Response size</t>
+          <t>A hash of the client's IP</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -1193,12 +1193,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>The order requests arrive - whose turn is it</t>
+          <t>Whose turn it is in a fixed rotation</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>One counter: servers[i++ % N]. It ignores how long each request takes - a 3 s export and a 5 ms health check are both “one turn”.</t>
+          <t>All four are real load balancing criteria, which is the trap: B is least connections, C is weighted round robin, D is IP hash. Round robin is one counter, servers[i++ % N], and knows only the order requests arrive - so a 3 s export and a 5 ms health check are both “one turn”.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Q15 distractors things an L4 balancer really does
"Preserve the client IP" and "hold a static IP" read as L4 strengths, so the
question was answerable without knowing why retry is L7-only. All three
distractors are now features L4 genuinely provides - SNI-based domain routing,
TLS termination on an NLB, health-check ejection - leaving the buffered retry
as the only true answer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2zDpHEjjhiN7Qvobfiizh
</commit_message>
<xml_diff>
--- a/kahoot-export/load-balancing-kahoot-15.xlsx
+++ b/kahoot-export/load-balancing-kahoot-15.xlsx
@@ -858,7 +858,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Preserve the client IP</t>
+          <t>Route traffic by domain name</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Hold a static IP</t>
+          <t>Eject a failing backend from the pool</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>The L7 proxy still holds the request bytes in memory, so it can write them to a second pod. L4 forwards each packet and forgets it, so there is nothing to replay. An NLB with a TLS listener does terminate TLS, which is what makes that option tempting.</t>
+          <t>Every option is a real balancer feature and L4 does three of them: it routes per domain by reading SNI in the clear, an NLB with a TLS listener terminates TLS, and health checks eject backends at both layers. Only the retry needs the request held in memory - L7 keeps a copy and can write it to a second pod, while L4 forwards each packet and forgets it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make Q20 distractors true facts that are not the reason
"The client cancels it" and "the health check fails" were obviously wrong.
The three distractors are now statements the deck actually makes - the 640 MB
buffer math, the ALB's 60 s idle timeout, the plaintext hop to the pod - so
the question turns on which one explains the lost retry rather than which one
sounds real.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D2zDpHEjjhiN7Qvobfiizh
</commit_message>
<xml_diff>
--- a/kahoot-export/load-balancing-kahoot-15.xlsx
+++ b/kahoot-export/load-balancing-kahoot-15.xlsx
@@ -924,17 +924,17 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>The client cancels it</t>
+          <t>10,000 concurrent requests at 64 KB would need 640 MB</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>The health check fails</t>
+          <t>It hits the 60 s idle timeout before the upload finishes</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Re-encryption to the pod drops it</t>
+          <t>The hop to the pod is plaintext, so the bytes are gone</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Retries exist only because the request sits in the proxy's memory. 10,000 concurrent requests x 64 KB is already 640 MB, so every balancer caps what it will buffer. Over the cap it streams the bytes straight through and retries quietly stop working.</t>
+          <t>B, C and D are all true statements from the deck, and none of them is the reason. 640 MB is why the cap exists, not why retries stop. 60 s is the ALB's default idle timeout. The hop to the pod really is plaintext unless you re-encrypt. Retries work only because the proxy still holds the request: over the cap it stops keeping a copy and streams the bytes straight through, so there is nothing left to re-send.</t>
         </is>
       </c>
     </row>

</xml_diff>